<commit_message>
chore(PC-001): one branch for all platform work; features ship with their companions
Founder decision 2026-09-26: all tasks on platform-completion, merged into main only on the
founder's word; commits as sanjeetji. AGENTS.md and the queue README say so, and a feature
now includes its obvious companions (R-591 covers forgot/reset password, not only login).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/Platform_Completion/OmniStackAI_Master_Tasks.xlsx
+++ b/R_&_D/Platform_Completion/OmniStackAI_Master_Tasks.xlsx
@@ -1092,7 +1092,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Login and register for the Go backend</t>
+          <t>Complete auth for the Go backend: register, login, logout, me, forgot password, reset password</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -1119,7 +1119,7 @@
       <c r="I7" s="3" t="inlineStr"/>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>A Go app with auth has no way for a real user to sign in.</t>
+          <t>A Go app with auth has no way for a real user to sign in. Parity with the Python backend's auth (R-461, R-463), companions included.</t>
         </is>
       </c>
     </row>
@@ -10945,7 +10945,7 @@
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>Login and register for the Go backend</t>
+          <t>Complete auth for the Go backend: register, login, logout, me, forgot password, reset password</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
@@ -10977,7 +10977,7 @@
       <c r="I104" s="3" t="inlineStr"/>
       <c r="J104" s="3" t="inlineStr">
         <is>
-          <t>A Go app with auth has no way for a real user to sign in.</t>
+          <t>A Go app with auth has no way for a real user to sign in. Parity with the Python backend's auth (R-461, R-463), companions included.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(PC-006): preview starts in half the time; model navigation can no longer break pages
PC-006 stays In Progress: speed half done, first-screen visual quality next.

- Generated Python APIs link to one shared, pre-compiled environment per
  requirements set instead of creating a venv and pip-installing on every
  preview; warmed at platform start.
- API, web, admin and mobile readiness are probed together every 0.25 s,
  not one after another every 1 s.
- Preview start 17.7 s -> 9.6 s; live prompt -> running app 12-15 s on Groq
  (was 18-26 s).
- Fixed: screen navigation written as objects rendered as broken links and
  uncompilable pages; links to missing screens are dropped.
- Generated .gitignore ignores .venv (a symlink), not only .venv/.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/Platform_Completion/OmniStackAI_Master_Tasks.xlsx
+++ b/R_&_D/Platform_Completion/OmniStackAI_Master_Tasks.xlsx
@@ -1399,7 +1399,7 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>R-558 fixed the design system; still needs speed-to-first-screen and visual quality. From specs/table-stakes/01 and the buildout 'intent card' idea. Measured in PC-084: plan 20-29 s (model) and preview start ~14 s are the stages to cut; model-written pages cost ~80 s and their admin page failed to compile, so the repair loop must cover the admin app before model-written pages return to the default path.</t>
+          <t>R-558 fixed the design system; still needs speed-to-first-screen and visual quality. From specs/table-stakes/01 and the buildout 'intent card' idea. Measured in PC-084: plan 20-29 s (model) and preview start ~14 s are the stages to cut; model-written pages cost ~80 s and their admin page failed to compile, so the repair loop must cover the admin app before model-written pages return to the default path. Speed half done 2026-09-26: preview start 17.7 -&gt; 9.6 s (shared warm API environment, surfaces probed together), live prompt -&gt; running app 12-15 s on Groq; fixed model navigation objects breaking pages. Left: visual quality of the first screen; starting the preview during verification (~5 s) once node_modules are not shared.</t>
         </is>
       </c>
     </row>
@@ -6407,7 +6407,7 @@
       <c r="I2" s="3" t="inlineStr"/>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>R-558 fixed the design system; still needs speed-to-first-screen and visual quality. From specs/table-stakes/01 and the buildout 'intent card' idea. Measured in PC-084: plan 20-29 s (model) and preview start ~14 s are the stages to cut; model-written pages cost ~80 s and their admin page failed to compile, so the repair loop must cover the admin app before model-written pages return to the default path.</t>
+          <t>R-558 fixed the design system; still needs speed-to-first-screen and visual quality. From specs/table-stakes/01 and the buildout 'intent card' idea. Measured in PC-084: plan 20-29 s (model) and preview start ~14 s are the stages to cut; model-written pages cost ~80 s and their admin page failed to compile, so the repair loop must cover the admin app before model-written pages return to the default path. Speed half done 2026-09-26: preview start 17.7 -&gt; 9.6 s (shared warm API environment, surfaces probed together), live prompt -&gt; running app 12-15 s on Groq; fixed model navigation objects breaking pages. Left: visual quality of the first screen; starting the preview during verification (~5 s) once node_modules are not shared.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(R-567): live proof with real Stripe and Razorpay test accounts
Bazaar Lite took a real test-mode payment through each provider: webhook
verified, seller credited 90%, refund made through the provider, books balanced.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/Platform_Completion/OmniStackAI_Master_Tasks.xlsx
+++ b/R_&_D/Platform_Completion/OmniStackAI_Master_Tasks.xlsx
@@ -3181,7 +3181,7 @@
       </c>
       <c r="J52" s="3" t="inlineStr">
         <is>
-          <t>R-512 gives Stripe/Razorpay checkout; this is the ledger. Done 2026-10-01: a `money` capability; every backend gets server-priced checkout, a double-entry ledger, commission splits, refunds and payouts, mock offline and verified Stripe/Razorpay webhooks. Real provider accounts are PC-070/PC-071; the screens are PC-113.</t>
+          <t>R-512 gives Stripe/Razorpay checkout; this is the ledger. Done 2026-10-01: a `money` capability; every backend gets server-priced checkout, a double-entry ledger, commission splits, refunds and payouts, mock offline and verified Stripe/Razorpay webhooks. Real provider accounts are PC-070/PC-071; the screens are PC-113. Proved with real test-mode accounts 2026-10-01 on the console-built Bazaar Lite: Stripe (card, webhook via the Stripe CLI) and Razorpay (netbanking, webhook via a tunnel) each took ₹799, credited the seller ₹719.10 and refunded ₹100 through the provider.</t>
         </is>
       </c>
     </row>
@@ -6835,7 +6835,7 @@
       </c>
       <c r="J131" s="3" t="inlineStr">
         <is>
-          <t>Publish to a real URL, a real payment, a real email, EAS/store uploads to both stores.</t>
+          <t>Publish to a real URL, a real payment, a real email, EAS/store uploads to both stores. Payments in test mode done 2026-10-01 (Stripe and Razorpay, see R-567); live-mode keys remain.</t>
         </is>
       </c>
     </row>
@@ -14659,7 +14659,7 @@
       <c r="I166" s="3" t="inlineStr"/>
       <c r="J166" s="3" t="inlineStr">
         <is>
-          <t>Publish to a real URL, a real payment, a real email, EAS/store uploads to both stores.</t>
+          <t>Publish to a real URL, a real payment, a real email, EAS/store uploads to both stores. Payments in test mode done 2026-10-01 (Stripe and Razorpay, see R-567); live-mode keys remain.</t>
         </is>
       </c>
     </row>
@@ -39243,7 +39243,7 @@
       </c>
       <c r="J726" s="3" t="inlineStr">
         <is>
-          <t>R-512 gives Stripe/Razorpay checkout; this is the ledger. Done 2026-10-01: a `money` capability; every backend gets server-priced checkout, a double-entry ledger, commission splits, refunds and payouts, mock offline and verified Stripe/Razorpay webhooks. Real provider accounts are PC-070/PC-071; the screens are PC-113.</t>
+          <t>R-512 gives Stripe/Razorpay checkout; this is the ledger. Done 2026-10-01: a `money` capability; every backend gets server-priced checkout, a double-entry ledger, commission splits, refunds and payouts, mock offline and verified Stripe/Razorpay webhooks. Real provider accounts are PC-070/PC-071; the screens are PC-113. Proved with real test-mode accounts 2026-10-01 on the console-built Bazaar Lite: Stripe (card, webhook via the Stripe CLI) and Razorpay (netbanking, webhook via a tunnel) each took ₹799, credited the seller ₹719.10 and refunded ₹100 through the provider.</t>
         </is>
       </c>
     </row>

</xml_diff>